<commit_message>
Updated National Schematron Rules Comparison (v3.4.0 to v3.5.0) for v3.5.0.250403CP5.
</commit_message>
<xml_diff>
--- a/Schematron/documentation/Schematron_3.4.0_3.5.0_Comparison.xlsx
+++ b/Schematron/documentation/Schematron_3.4.0_3.5.0_Comparison.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Josh\Documents\NEMSIS TAC\Repository\nemsis\Schematron\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Josh\Documents\NEMSIS TAC\Repository\nemsis_public\Schematron\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20676D51-0773-42CF-81B1-CC9508344358}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2ADF1B2-0C50-4D56-BA2A-F7E7740364F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{EFB0DDD4-CF85-4C10-9AFB-9B88D9ECAAEF}"/>
   </bookViews>
@@ -760,9 +760,6 @@
     <t>nemSch_e060</t>
   </si>
   <si>
-    <t>nemSch_e061</t>
-  </si>
-  <si>
     <t>nemSch_e062</t>
   </si>
   <si>
@@ -1399,9 +1396,6 @@
     <t>Patient's Home ZIP Code should be recorded when Patient Evaluation/Care is "Patient Evaluated and Care Provided".</t>
   </si>
   <si>
-    <t>Gender should be recorded when Patient Evaluation/Care is "Patient Evaluated and Care Provided".</t>
-  </si>
-  <si>
     <t>Race should be recorded when Patient Evaluation/Care is "Patient Evaluated and Care Provided".</t>
   </si>
   <si>
@@ -1909,13 +1903,19 @@
     <t>Trauma Triage Criteria (Moderate Risk for Serious Injury) should only be recorded when Possible Injury is "Yes".</t>
   </si>
   <si>
-    <t>National Schematron Rules Comparison for EMSDataSet - March 17, 2023</t>
-  </si>
-  <si>
-    <t>3.5.0.230317CP4</t>
-  </si>
-  <si>
-    <t>National Schematron Rules Comparison for DEMDataSet - March 17, 2023</t>
+    <t>National Schematron Rules Comparison for DEMDataSet</t>
+  </si>
+  <si>
+    <t>3.5.0.250403CP5</t>
+  </si>
+  <si>
+    <t>National Schematron Rules Comparison for EMSDataSet</t>
+  </si>
+  <si>
+    <t>nemSch_e193</t>
+  </si>
+  <si>
+    <t>Sex should be recorded when Patient Evaluation/Care is "Patient Evaluated and Care Provided".</t>
   </si>
 </sst>
 </file>
@@ -1977,7 +1977,91 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="31">
+  <dxfs count="36">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -2020,27 +2104,6 @@
       <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2066,34 +2129,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -2147,10 +2182,10 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="TableStyleMedium4 2" pivot="0" count="4" xr9:uid="{C5EDC0DC-20C1-4753-97CF-DF11B24525E0}">
-      <tableStyleElement type="wholeTable" dxfId="30"/>
-      <tableStyleElement type="headerRow" dxfId="29"/>
-      <tableStyleElement type="firstRowStripe" dxfId="28"/>
-      <tableStyleElement type="secondRowStripe" dxfId="27"/>
+      <tableStyleElement type="wholeTable" dxfId="35"/>
+      <tableStyleElement type="headerRow" dxfId="34"/>
+      <tableStyleElement type="firstRowStripe" dxfId="33"/>
+      <tableStyleElement type="secondRowStripe" dxfId="32"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -2171,41 +2206,41 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D5FB1F5A-F1E9-47F6-9AE4-2715FA1AD725}" name="DEMDataSet" displayName="DEMDataSet" ref="A3:G25" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D5FB1F5A-F1E9-47F6-9AE4-2715FA1AD725}" name="DEMDataSet" displayName="DEMDataSet" ref="A3:G25" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
   <autoFilter ref="A3:G25" xr:uid="{D5FB1F5A-F1E9-47F6-9AE4-2715FA1AD725}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{818C128E-3E91-44CB-BDC2-CEE48E82002C}" name="3.4 ID" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{EC5E3CC2-931F-4F0B-AF7C-D89978263779}" name="3.4 Level" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{2AE98681-7191-400C-A1BB-F4A87B16587B}" name="3.4 Message" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{6515116D-5BF3-4EA2-A88E-266F809C488A}" name="-" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{8FE0A1BD-6739-4485-9956-84D3D8EE8C0F}" name="3.5 ID" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{CE2E930A-1FEE-4B87-82B2-ACD8CBCD57E2}" name="3.5 Level" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{ED19B31C-FD36-408B-8438-FBF75CBC535A}" name="3.5 Message" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{818C128E-3E91-44CB-BDC2-CEE48E82002C}" name="3.4 ID" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{EC5E3CC2-931F-4F0B-AF7C-D89978263779}" name="3.4 Level" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{2AE98681-7191-400C-A1BB-F4A87B16587B}" name="3.4 Message" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{6515116D-5BF3-4EA2-A88E-266F809C488A}" name="-" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{8FE0A1BD-6739-4485-9956-84D3D8EE8C0F}" name="3.5 ID" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{CE2E930A-1FEE-4B87-82B2-ACD8CBCD57E2}" name="3.5 Level" dataDxfId="24"/>
+    <tableColumn id="7" xr3:uid="{ED19B31C-FD36-408B-8438-FBF75CBC535A}" name="3.5 Message" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4 2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8C501FD1-013C-47C7-A243-7EF4752BD2F0}" name="EMSDataSet" displayName="EMSDataSet" ref="A3:G199" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7">
-  <autoFilter ref="A3:G199" xr:uid="{8C501FD1-013C-47C7-A243-7EF4752BD2F0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8C501FD1-013C-47C7-A243-7EF4752BD2F0}" name="EMSDataSet" displayName="EMSDataSet" ref="A3:G200" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19">
+  <autoFilter ref="A3:G200" xr:uid="{8C501FD1-013C-47C7-A243-7EF4752BD2F0}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{E40A4C59-3E85-43EC-80D4-06A76F43E07B}" name="3.4 ID" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{40C08B32-31C2-40E1-888B-9F302CE52BD0}" name="3.4 Level" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{5189CD8A-54FE-4A9B-8418-66C6E7C501BE}" name="3.4 Message" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{C283BDAA-022C-4DFA-A2CB-1131836708B9}" name="-" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{91B23EFB-DAB3-470B-8F24-35C725763D5F}" name="3.5 ID" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{B9DFE584-8591-4FE2-BDAC-2E27E531CDEC}" name="3.5 Level" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{4DE8F714-A13E-44A3-B722-6EB4CCB93F87}" name="3.5 Message" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{E40A4C59-3E85-43EC-80D4-06A76F43E07B}" name="3.4 ID" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{40C08B32-31C2-40E1-888B-9F302CE52BD0}" name="3.4 Level" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{5189CD8A-54FE-4A9B-8418-66C6E7C501BE}" name="3.4 Message" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{C283BDAA-022C-4DFA-A2CB-1131836708B9}" name="-" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{91B23EFB-DAB3-470B-8F24-35C725763D5F}" name="3.5 ID" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{B9DFE584-8591-4FE2-BDAC-2E27E531CDEC}" name="3.5 Level" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{4DE8F714-A13E-44A3-B722-6EB4CCB93F87}" name="3.5 Message" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4 2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2243,7 +2278,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2349,7 +2384,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2491,7 +2526,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2514,7 +2549,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>626</v>
+        <v>622</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -2530,32 +2565,32 @@
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="E2" s="4" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>373</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="2" t="s">
         <v>371</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -2566,7 +2601,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>0</v>
@@ -2575,7 +2610,7 @@
         <v>1</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -2586,7 +2621,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>0</v>
@@ -2595,7 +2630,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -2606,7 +2641,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>15</v>
@@ -2615,7 +2650,7 @@
         <v>5</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2626,7 +2661,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>16</v>
@@ -2635,7 +2670,7 @@
         <v>5</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2646,7 +2681,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>17</v>
@@ -2655,7 +2690,7 @@
         <v>1</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -2666,7 +2701,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -2688,7 +2723,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>21</v>
@@ -2697,7 +2732,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -2708,7 +2743,7 @@
         <v>1</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>22</v>
@@ -2717,7 +2752,7 @@
         <v>1</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2728,7 +2763,7 @@
         <v>1</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>23</v>
@@ -2737,7 +2772,7 @@
         <v>1</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2748,7 +2783,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>24</v>
@@ -2757,7 +2792,7 @@
         <v>1</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -2769,7 +2804,7 @@
         <v>1</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2781,7 +2816,7 @@
         <v>1</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -2792,7 +2827,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -2803,7 +2838,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2814,7 +2849,7 @@
         <v>5</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -2825,7 +2860,7 @@
         <v>5</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -2836,7 +2871,7 @@
         <v>5</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2847,7 +2882,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>32</v>
@@ -2856,7 +2891,7 @@
         <v>1</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
@@ -2867,7 +2902,7 @@
         <v>1</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2878,7 +2913,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2889,7 +2924,7 @@
         <v>1</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>
@@ -2898,24 +2933,14 @@
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="B4:B25">
-    <cfRule type="cellIs" dxfId="26" priority="3" operator="notEqual">
+  <conditionalFormatting sqref="B4:C25">
+    <cfRule type="cellIs" dxfId="10" priority="3" operator="notEqual">
       <formula>F4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F4:F25">
-    <cfRule type="cellIs" dxfId="25" priority="4" operator="notEqual">
+  <conditionalFormatting sqref="F4:G25">
+    <cfRule type="cellIs" dxfId="9" priority="4" operator="notEqual">
       <formula>B4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C4:C25">
-    <cfRule type="cellIs" dxfId="24" priority="2" operator="notEqual">
-      <formula>G4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G4:G25">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="notEqual">
-      <formula>C4</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2959,32 +2984,32 @@
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="E2" s="4" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>368</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>373</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>371</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -2995,7 +3020,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>0</v>
@@ -3004,7 +3029,7 @@
         <v>1</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3035,7 +3060,7 @@
         <v>1</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -3046,7 +3071,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>0</v>
@@ -3055,7 +3080,7 @@
         <v>1</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -3097,7 +3122,7 @@
         <v>5</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>181</v>
@@ -3106,7 +3131,7 @@
         <v>5</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3117,7 +3142,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>182</v>
@@ -3126,7 +3151,7 @@
         <v>5</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -3138,7 +3163,7 @@
         <v>5</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -3149,7 +3174,7 @@
         <v>5</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -3160,7 +3185,7 @@
         <v>5</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -3171,7 +3196,7 @@
         <v>5</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>186</v>
@@ -3180,7 +3205,7 @@
         <v>5</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -3191,7 +3216,7 @@
         <v>5</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>187</v>
@@ -3200,7 +3225,7 @@
         <v>5</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -3211,7 +3236,7 @@
         <v>5</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>188</v>
@@ -3220,7 +3245,7 @@
         <v>5</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3231,7 +3256,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>189</v>
@@ -3240,7 +3265,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3251,7 +3276,7 @@
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>190</v>
@@ -3260,7 +3285,7 @@
         <v>1</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -3271,7 +3296,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>191</v>
@@ -3280,7 +3305,7 @@
         <v>1</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3291,7 +3316,7 @@
         <v>1</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>192</v>
@@ -3300,7 +3325,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3311,7 +3336,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>193</v>
@@ -3320,7 +3345,7 @@
         <v>1</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3331,7 +3356,7 @@
         <v>1</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>194</v>
@@ -3340,7 +3365,7 @@
         <v>1</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3351,7 +3376,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>195</v>
@@ -3360,7 +3385,7 @@
         <v>1</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3371,7 +3396,7 @@
         <v>1</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>196</v>
@@ -3380,7 +3405,7 @@
         <v>1</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3391,7 +3416,7 @@
         <v>1</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>197</v>
@@ -3400,7 +3425,7 @@
         <v>1</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -3411,7 +3436,7 @@
         <v>1</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>198</v>
@@ -3420,7 +3445,7 @@
         <v>1</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3431,7 +3456,7 @@
         <v>1</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>199</v>
@@ -3440,7 +3465,7 @@
         <v>1</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -3451,7 +3476,7 @@
         <v>1</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>200</v>
@@ -3460,7 +3485,7 @@
         <v>1</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3471,7 +3496,7 @@
         <v>1</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>201</v>
@@ -3480,7 +3505,7 @@
         <v>1</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3491,7 +3516,7 @@
         <v>1</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>202</v>
@@ -3500,7 +3525,7 @@
         <v>1</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3511,7 +3536,7 @@
         <v>1</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>203</v>
@@ -3520,7 +3545,7 @@
         <v>1</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3531,7 +3556,7 @@
         <v>1</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>204</v>
@@ -3540,7 +3565,7 @@
         <v>1</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -3551,7 +3576,7 @@
         <v>1</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>205</v>
@@ -3560,7 +3585,7 @@
         <v>1</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3571,7 +3596,7 @@
         <v>1</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>206</v>
@@ -3580,7 +3605,7 @@
         <v>1</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3591,7 +3616,7 @@
         <v>1</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>207</v>
@@ -3600,7 +3625,7 @@
         <v>1</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3611,7 +3636,7 @@
         <v>1</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>208</v>
@@ -3620,7 +3645,7 @@
         <v>1</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3631,7 +3656,7 @@
         <v>1</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>209</v>
@@ -3640,7 +3665,7 @@
         <v>1</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -3651,7 +3676,7 @@
         <v>1</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>210</v>
@@ -3660,7 +3685,7 @@
         <v>1</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3671,7 +3696,7 @@
         <v>1</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>211</v>
@@ -3680,7 +3705,7 @@
         <v>1</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3691,7 +3716,7 @@
         <v>1</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>212</v>
@@ -3700,7 +3725,7 @@
         <v>1</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3711,7 +3736,7 @@
         <v>1</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>213</v>
@@ -3720,7 +3745,7 @@
         <v>1</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3731,7 +3756,7 @@
         <v>1</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>214</v>
@@ -3740,7 +3765,7 @@
         <v>1</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3751,7 +3776,7 @@
         <v>1</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>215</v>
@@ -3760,7 +3785,7 @@
         <v>1</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -3771,7 +3796,7 @@
         <v>1</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>216</v>
@@ -3780,7 +3805,7 @@
         <v>1</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3791,7 +3816,7 @@
         <v>1</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>217</v>
@@ -3800,7 +3825,7 @@
         <v>1</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3811,7 +3836,7 @@
         <v>1</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>218</v>
@@ -3820,7 +3845,7 @@
         <v>1</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3831,7 +3856,7 @@
         <v>1</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>219</v>
@@ -3840,7 +3865,7 @@
         <v>1</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3851,7 +3876,7 @@
         <v>1</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>220</v>
@@ -3860,7 +3885,7 @@
         <v>1</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3871,7 +3896,7 @@
         <v>1</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>221</v>
@@ -3880,7 +3905,7 @@
         <v>1</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3891,7 +3916,7 @@
         <v>1</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>222</v>
@@ -3900,7 +3925,7 @@
         <v>1</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3911,7 +3936,7 @@
         <v>1</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>223</v>
@@ -3920,7 +3945,7 @@
         <v>1</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3931,7 +3956,7 @@
         <v>1</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3942,7 +3967,7 @@
         <v>1</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>225</v>
@@ -3951,7 +3976,7 @@
         <v>1</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3962,7 +3987,7 @@
         <v>1</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>226</v>
@@ -3971,7 +3996,7 @@
         <v>1</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3982,7 +4007,7 @@
         <v>1</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>227</v>
@@ -3991,7 +4016,7 @@
         <v>1</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4002,7 +4027,7 @@
         <v>1</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>228</v>
@@ -4011,7 +4036,7 @@
         <v>1</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4022,7 +4047,7 @@
         <v>1</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>229</v>
@@ -4031,7 +4056,7 @@
         <v>1</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4042,7 +4067,7 @@
         <v>1</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>230</v>
@@ -4051,7 +4076,7 @@
         <v>1</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4062,7 +4087,7 @@
         <v>1</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>231</v>
@@ -4071,7 +4096,7 @@
         <v>1</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4082,7 +4107,7 @@
         <v>1</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>232</v>
@@ -4091,7 +4116,7 @@
         <v>1</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4102,7 +4127,7 @@
         <v>1</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>233</v>
@@ -4111,7 +4136,7 @@
         <v>1</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4122,7 +4147,7 @@
         <v>1</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4133,7 +4158,7 @@
         <v>1</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>235</v>
@@ -4142,7 +4167,7 @@
         <v>1</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4153,7 +4178,7 @@
         <v>1</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>236</v>
@@ -4162,7 +4187,7 @@
         <v>1</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4173,7 +4198,7 @@
         <v>1</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>237</v>
@@ -4182,7 +4207,7 @@
         <v>1</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4193,7 +4218,7 @@
         <v>1</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>238</v>
@@ -4202,7 +4227,7 @@
         <v>1</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4213,7 +4238,7 @@
         <v>1</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>239</v>
@@ -4222,7 +4247,7 @@
         <v>1</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4233,7 +4258,7 @@
         <v>1</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>240</v>
@@ -4242,7 +4267,7 @@
         <v>1</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4253,16 +4278,7 @@
         <v>1</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>598</v>
-      </c>
-      <c r="E70" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="F70" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G70" s="2" t="s">
-        <v>454</v>
+        <v>596</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4273,16 +4289,16 @@
         <v>1</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4293,16 +4309,16 @@
         <v>1</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4313,16 +4329,16 @@
         <v>1</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F73" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
@@ -4333,16 +4349,16 @@
         <v>1</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F74" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4353,28 +4369,28 @@
         <v>1</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F75" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C76" s="1"/>
       <c r="E76" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F76" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4385,16 +4401,16 @@
         <v>1</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F77" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4405,16 +4421,16 @@
         <v>1</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F78" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4425,49 +4441,49 @@
         <v>1</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F79" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="E80" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F80" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="E81" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F81" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="E82" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F82" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
@@ -4478,27 +4494,27 @@
         <v>1</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F83" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="E84" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F84" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4509,16 +4525,16 @@
         <v>1</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F85" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4529,16 +4545,16 @@
         <v>1</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F86" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4549,16 +4565,16 @@
         <v>1</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F87" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4569,16 +4585,16 @@
         <v>1</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F88" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4589,16 +4605,16 @@
         <v>1</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F89" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4609,16 +4625,16 @@
         <v>1</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F90" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4629,16 +4645,16 @@
         <v>1</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F91" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4649,16 +4665,16 @@
         <v>1</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F92" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4669,62 +4685,62 @@
         <v>1</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F93" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C94" s="1"/>
       <c r="E94" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F94" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C95" s="1"/>
       <c r="E95" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F95" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="E96" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F96" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="E97" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F97" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4735,16 +4751,16 @@
         <v>1</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F98" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4755,16 +4771,16 @@
         <v>1</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F99" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4775,16 +4791,16 @@
         <v>1</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F100" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4795,16 +4811,16 @@
         <v>1</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F101" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4815,16 +4831,16 @@
         <v>1</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F102" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G102" s="2" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4835,16 +4851,16 @@
         <v>1</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F103" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4855,16 +4871,16 @@
         <v>1</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F104" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G104" s="2" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4875,16 +4891,16 @@
         <v>1</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F105" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="106" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4895,16 +4911,16 @@
         <v>1</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F106" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G106" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
     </row>
     <row r="107" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4915,16 +4931,16 @@
         <v>1</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F107" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G107" s="2" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
     </row>
     <row r="108" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4935,16 +4951,16 @@
         <v>1</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F108" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G108" s="2" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
     </row>
     <row r="109" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4955,16 +4971,16 @@
         <v>1</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F109" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G109" s="2" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
     </row>
     <row r="110" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4975,16 +4991,16 @@
         <v>1</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F110" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G110" s="2" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
     </row>
     <row r="111" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4995,16 +5011,16 @@
         <v>1</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F111" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G111" s="2" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
     </row>
     <row r="112" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5015,7 +5031,7 @@
         <v>1</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
     </row>
     <row r="113" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5026,7 +5042,7 @@
         <v>1</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="G113" s="1"/>
     </row>
@@ -5038,16 +5054,16 @@
         <v>1</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F114" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G114" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="115" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5058,16 +5074,16 @@
         <v>1</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F115" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G115" s="2" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
     </row>
     <row r="116" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5078,16 +5094,16 @@
         <v>1</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F116" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="117" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5098,16 +5114,16 @@
         <v>1</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F117" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G117" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -5118,28 +5134,28 @@
         <v>1</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="E118" s="1" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F118" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G118" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="119" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C119" s="1"/>
       <c r="E119" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F119" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G119" s="2" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
     </row>
     <row r="120" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5150,16 +5166,16 @@
         <v>1</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F120" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G120" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="121" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5170,16 +5186,16 @@
         <v>1</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F121" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G121" s="2" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="122" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5190,16 +5206,16 @@
         <v>1</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F122" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G122" s="2" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
     </row>
     <row r="123" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5210,7 +5226,7 @@
         <v>1</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
     </row>
     <row r="124" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5221,16 +5237,16 @@
         <v>1</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="E124" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F124" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G124" s="2" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
     </row>
     <row r="125" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -5241,16 +5257,16 @@
         <v>1</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="E125" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F125" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G125" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
     </row>
     <row r="126" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5261,27 +5277,27 @@
         <v>1</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="E126" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F126" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G126" s="2" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="E127" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F127" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G127" s="2" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
     </row>
     <row r="128" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5292,86 +5308,86 @@
         <v>1</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="E128" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F128" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G128" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
     </row>
     <row r="129" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C129" s="1"/>
       <c r="E129" s="1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F129" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G129" s="2" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
     </row>
     <row r="130" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C130" s="1"/>
       <c r="E130" s="1" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F130" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="131" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="E131" s="1" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F131" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G131" s="2" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
     </row>
     <row r="132" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C132" s="1"/>
       <c r="E132" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F132" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G132" s="2" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
     </row>
     <row r="133" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="E133" s="1" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F133" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G133" s="2" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
     </row>
     <row r="134" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C134" s="1"/>
       <c r="E134" s="1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F134" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G134" s="2" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
     </row>
     <row r="135" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5382,16 +5398,16 @@
         <v>1</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="E135" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F135" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G135" s="2" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
     </row>
     <row r="136" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5402,16 +5418,16 @@
         <v>1</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="E136" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F136" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G136" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="137" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5422,16 +5438,16 @@
         <v>1</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="E137" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F137" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G137" s="2" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
     </row>
     <row r="138" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5442,16 +5458,16 @@
         <v>1</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="E138" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F138" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G138" s="2" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="139" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5462,16 +5478,16 @@
         <v>1</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="E139" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F139" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G139" s="2" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
     </row>
     <row r="140" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5482,16 +5498,16 @@
         <v>1</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="E140" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F140" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G140" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="141" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5502,64 +5518,64 @@
         <v>1</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="E141" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F141" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G141" s="2" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="142" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C142" s="1"/>
       <c r="E142" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F142" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G142" s="2" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
     </row>
     <row r="143" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C143" s="1"/>
       <c r="E143" s="1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F143" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G143" s="2" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
     </row>
     <row r="144" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C144" s="1"/>
       <c r="E144" s="1" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F144" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G144" s="2" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
     </row>
     <row r="145" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C145" s="1"/>
       <c r="E145" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F145" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G145" s="2" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
     </row>
     <row r="146" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5570,16 +5586,16 @@
         <v>1</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="E146" s="1" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F146" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G146" s="2" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="147" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5590,16 +5606,16 @@
         <v>1</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="E147" s="1" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F147" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G147" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="148" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -5610,16 +5626,16 @@
         <v>1</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="E148" s="1" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F148" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G148" s="2" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="149" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5630,16 +5646,16 @@
         <v>1</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="E149" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F149" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G149" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="150" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5650,16 +5666,16 @@
         <v>1</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="E150" s="1" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F150" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G150" s="2" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="151" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5670,16 +5686,16 @@
         <v>1</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="E151" s="1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F151" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G151" s="2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
     <row r="152" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5690,16 +5706,16 @@
         <v>1</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="E152" s="1" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="F152" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G152" s="2" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
     </row>
     <row r="153" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5710,75 +5726,75 @@
         <v>1</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="E153" s="1" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F153" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G153" s="2" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
     </row>
     <row r="154" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C154" s="1"/>
       <c r="E154" s="1" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="F154" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G154" s="2" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
     </row>
     <row r="155" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C155" s="1"/>
       <c r="E155" s="1" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F155" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G155" s="2" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="156" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C156" s="1"/>
       <c r="E156" s="1" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F156" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G156" s="2" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
     </row>
     <row r="157" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C157" s="1"/>
       <c r="E157" s="1" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F157" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G157" s="2" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
     </row>
     <row r="158" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="E158" s="1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="F158" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G158" s="2" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
     </row>
     <row r="159" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5789,16 +5805,16 @@
         <v>1</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="E159" s="1" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="F159" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G159" s="2" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
     </row>
     <row r="160" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5809,28 +5825,28 @@
         <v>1</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="E160" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="F160" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G160" s="2" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
     </row>
     <row r="161" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C161" s="1"/>
       <c r="E161" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F161" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G161" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
     </row>
     <row r="162" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5841,16 +5857,16 @@
         <v>1</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="E162" s="1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F162" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G162" s="2" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="163" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5861,16 +5877,16 @@
         <v>1</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="E163" s="1" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F163" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G163" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
     </row>
     <row r="164" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5881,16 +5897,16 @@
         <v>1</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="E164" s="1" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F164" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G164" s="2" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
     </row>
     <row r="165" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5901,16 +5917,16 @@
         <v>1</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="E165" s="1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F165" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G165" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
     </row>
     <row r="166" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5921,16 +5937,16 @@
         <v>1</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="E166" s="1" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F166" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G166" s="2" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
     </row>
     <row r="167" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5941,16 +5957,16 @@
         <v>1</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="E167" s="1" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F167" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G167" s="2" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="168" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5961,16 +5977,16 @@
         <v>1</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="E168" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F168" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G168" s="2" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
     </row>
     <row r="169" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5981,27 +5997,27 @@
         <v>1</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="E169" s="1" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F169" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G169" s="2" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
     </row>
     <row r="170" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="E170" s="1" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F170" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G170" s="2" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
     </row>
     <row r="171" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6012,16 +6028,16 @@
         <v>1</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="E171" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F171" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G171" s="2" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
     </row>
     <row r="172" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6032,16 +6048,16 @@
         <v>1</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="E172" s="1" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F172" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G172" s="2" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
     </row>
     <row r="173" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -6052,16 +6068,16 @@
         <v>1</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="E173" s="1" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F173" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G173" s="2" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
     </row>
     <row r="174" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6072,16 +6088,16 @@
         <v>1</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="E174" s="1" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F174" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G174" s="2" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="175" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6092,28 +6108,28 @@
         <v>1</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="E175" s="1" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F175" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G175" s="2" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="176" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C176" s="1"/>
       <c r="E176" s="1" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="F176" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G176" s="2" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="177" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6124,28 +6140,28 @@
         <v>1</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="E177" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F177" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G177" s="2" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="178" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C178" s="1"/>
       <c r="E178" s="1" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F178" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G178" s="2" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="179" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6156,16 +6172,16 @@
         <v>1</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E179" s="1" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="F179" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G179" s="2" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="180" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6176,16 +6192,16 @@
         <v>1</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="E180" s="1" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F180" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G180" s="2" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="181" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6196,16 +6212,16 @@
         <v>1</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="E181" s="1" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F181" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G181" s="2" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="182" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6216,7 +6232,7 @@
         <v>1</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="183" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6227,16 +6243,16 @@
         <v>1</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="E183" s="1" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="F183" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G183" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="184" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6247,16 +6263,16 @@
         <v>1</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="E184" s="1" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="F184" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G184" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="185" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -6267,27 +6283,27 @@
         <v>1</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="E185" s="1" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="F185" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G185" s="2" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="186" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="E186" s="1" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="F186" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G186" s="2" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="187" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6298,16 +6314,16 @@
         <v>1</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="E187" s="1" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F187" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G187" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
     </row>
     <row r="188" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6318,16 +6334,16 @@
         <v>1</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="E188" s="1" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="F188" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G188" s="2" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
     </row>
     <row r="189" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6338,16 +6354,16 @@
         <v>1</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="E189" s="1" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="F189" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G189" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
     </row>
     <row r="190" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -6358,16 +6374,16 @@
         <v>1</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="E190" s="1" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="F190" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G190" s="2" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
     </row>
     <row r="191" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -6378,116 +6394,125 @@
         <v>1</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="E191" s="1" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="F191" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G191" s="2" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
     </row>
     <row r="192" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C192" s="1"/>
       <c r="E192" s="1" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F192" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G192" s="2" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
     </row>
     <row r="193" spans="3:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C193" s="1"/>
       <c r="E193" s="1" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="F193" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G193" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
     </row>
     <row r="194" spans="3:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C194" s="1"/>
       <c r="E194" s="1" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F194" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G194" s="2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="195" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C195" s="1"/>
       <c r="E195" s="1" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F195" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G195" s="2" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
     </row>
     <row r="196" spans="3:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C196" s="1"/>
       <c r="E196" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F196" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G196" s="2" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
     </row>
     <row r="197" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C197" s="1"/>
       <c r="E197" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F197" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G197" s="2" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
     </row>
     <row r="198" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C198" s="1"/>
       <c r="E198" s="1" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="F198" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G198" s="2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
     </row>
     <row r="199" spans="3:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C199" s="1"/>
       <c r="E199" s="1" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F199" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G199" s="2" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="200" spans="3:7" x14ac:dyDescent="0.3">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="200" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C200" s="1"/>
+      <c r="E200" s="1" t="s">
+        <v>625</v>
+      </c>
+      <c r="F200" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G200" s="2" t="s">
+        <v>626</v>
+      </c>
     </row>
     <row r="201" spans="3:7" x14ac:dyDescent="0.3">
       <c r="C201" s="1"/>
@@ -6537,19 +6562,14 @@
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B4:C199">
-    <cfRule type="cellIs" dxfId="13" priority="4" operator="notEqual">
+  <conditionalFormatting sqref="B4:C200">
+    <cfRule type="cellIs" dxfId="4" priority="4" operator="notEqual">
       <formula>F4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F4:G26 F28:G199 F27">
-    <cfRule type="cellIs" dxfId="12" priority="5" operator="notEqual">
+  <conditionalFormatting sqref="F4:G200">
+    <cfRule type="cellIs" dxfId="3" priority="5" operator="notEqual">
       <formula>B4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G27">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="notEqual">
-      <formula>K27</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Schematron updates for v3.5.0.251001CP6.
</commit_message>
<xml_diff>
--- a/Schematron/documentation/Schematron_3.4.0_3.5.0_Comparison.xlsx
+++ b/Schematron/documentation/Schematron_3.4.0_3.5.0_Comparison.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Josh\Documents\NEMSIS TAC\Repository\nemsis_public\Schematron\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Josh\Documents\NEMSIS TAC\Repository\nemsis\Schematron\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2ADF1B2-0C50-4D56-BA2A-F7E7740364F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{981AC96C-BE3C-40E0-A37F-36734D4ECBCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{EFB0DDD4-CF85-4C10-9AFB-9B88D9ECAAEF}"/>
   </bookViews>
@@ -1903,19 +1903,19 @@
     <t>Trauma Triage Criteria (Moderate Risk for Serious Injury) should only be recorded when Possible Injury is "Yes".</t>
   </si>
   <si>
-    <t>National Schematron Rules Comparison for DEMDataSet</t>
-  </si>
-  <si>
-    <t>3.5.0.250403CP5</t>
-  </si>
-  <si>
-    <t>National Schematron Rules Comparison for EMSDataSet</t>
-  </si>
-  <si>
     <t>nemSch_e193</t>
   </si>
   <si>
     <t>Sex should be recorded when Patient Evaluation/Care is "Patient Evaluated and Care Provided".</t>
+  </si>
+  <si>
+    <t>National Schematron Rules Comparison for EMSDataSet - September 25, 2025</t>
+  </si>
+  <si>
+    <t>3.5.0.251001CP6</t>
+  </si>
+  <si>
+    <t>National Schematron Rules Comparison for DEMDataSet - September 25, 2025</t>
   </si>
 </sst>
 </file>
@@ -1977,63 +1977,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="36">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="28">
     <dxf>
       <fill>
         <patternFill>
@@ -2182,10 +2126,10 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="TableStyleMedium4 2" pivot="0" count="4" xr9:uid="{C5EDC0DC-20C1-4753-97CF-DF11B24525E0}">
-      <tableStyleElement type="wholeTable" dxfId="35"/>
-      <tableStyleElement type="headerRow" dxfId="34"/>
-      <tableStyleElement type="firstRowStripe" dxfId="33"/>
-      <tableStyleElement type="secondRowStripe" dxfId="32"/>
+      <tableStyleElement type="wholeTable" dxfId="27"/>
+      <tableStyleElement type="headerRow" dxfId="26"/>
+      <tableStyleElement type="firstRowStripe" dxfId="25"/>
+      <tableStyleElement type="secondRowStripe" dxfId="24"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -2206,32 +2150,32 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D5FB1F5A-F1E9-47F6-9AE4-2715FA1AD725}" name="DEMDataSet" displayName="DEMDataSet" ref="A3:G25" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D5FB1F5A-F1E9-47F6-9AE4-2715FA1AD725}" name="DEMDataSet" displayName="DEMDataSet" ref="A3:G25" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="A3:G25" xr:uid="{D5FB1F5A-F1E9-47F6-9AE4-2715FA1AD725}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{818C128E-3E91-44CB-BDC2-CEE48E82002C}" name="3.4 ID" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{EC5E3CC2-931F-4F0B-AF7C-D89978263779}" name="3.4 Level" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{2AE98681-7191-400C-A1BB-F4A87B16587B}" name="3.4 Message" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{6515116D-5BF3-4EA2-A88E-266F809C488A}" name="-" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{8FE0A1BD-6739-4485-9956-84D3D8EE8C0F}" name="3.5 ID" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{CE2E930A-1FEE-4B87-82B2-ACD8CBCD57E2}" name="3.5 Level" dataDxfId="24"/>
-    <tableColumn id="7" xr3:uid="{ED19B31C-FD36-408B-8438-FBF75CBC535A}" name="3.5 Message" dataDxfId="23"/>
+    <tableColumn id="1" xr3:uid="{818C128E-3E91-44CB-BDC2-CEE48E82002C}" name="3.4 ID" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{EC5E3CC2-931F-4F0B-AF7C-D89978263779}" name="3.4 Level" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{2AE98681-7191-400C-A1BB-F4A87B16587B}" name="3.4 Message" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{6515116D-5BF3-4EA2-A88E-266F809C488A}" name="-" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{8FE0A1BD-6739-4485-9956-84D3D8EE8C0F}" name="3.5 ID" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{CE2E930A-1FEE-4B87-82B2-ACD8CBCD57E2}" name="3.5 Level" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{ED19B31C-FD36-408B-8438-FBF75CBC535A}" name="3.5 Message" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4 2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8C501FD1-013C-47C7-A243-7EF4752BD2F0}" name="EMSDataSet" displayName="EMSDataSet" ref="A3:G200" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8C501FD1-013C-47C7-A243-7EF4752BD2F0}" name="EMSDataSet" displayName="EMSDataSet" ref="A3:G200" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11">
   <autoFilter ref="A3:G200" xr:uid="{8C501FD1-013C-47C7-A243-7EF4752BD2F0}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{E40A4C59-3E85-43EC-80D4-06A76F43E07B}" name="3.4 ID" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{40C08B32-31C2-40E1-888B-9F302CE52BD0}" name="3.4 Level" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{5189CD8A-54FE-4A9B-8418-66C6E7C501BE}" name="3.4 Message" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{C283BDAA-022C-4DFA-A2CB-1131836708B9}" name="-" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{91B23EFB-DAB3-470B-8F24-35C725763D5F}" name="3.5 ID" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{B9DFE584-8591-4FE2-BDAC-2E27E531CDEC}" name="3.5 Level" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{4DE8F714-A13E-44A3-B722-6EB4CCB93F87}" name="3.5 Message" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{E40A4C59-3E85-43EC-80D4-06A76F43E07B}" name="3.4 ID" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{40C08B32-31C2-40E1-888B-9F302CE52BD0}" name="3.4 Level" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{5189CD8A-54FE-4A9B-8418-66C6E7C501BE}" name="3.4 Message" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{C283BDAA-022C-4DFA-A2CB-1131836708B9}" name="-" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{91B23EFB-DAB3-470B-8F24-35C725763D5F}" name="3.5 ID" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{B9DFE584-8591-4FE2-BDAC-2E27E531CDEC}" name="3.5 Level" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{4DE8F714-A13E-44A3-B722-6EB4CCB93F87}" name="3.5 Message" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4 2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2549,7 +2493,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -2565,7 +2509,7 @@
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="E2" s="4" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
@@ -2934,12 +2878,12 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:C25">
-    <cfRule type="cellIs" dxfId="10" priority="3" operator="notEqual">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="notEqual">
       <formula>F4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F4:G25">
-    <cfRule type="cellIs" dxfId="9" priority="4" operator="notEqual">
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="notEqual">
       <formula>B4</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2984,7 +2928,7 @@
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="E2" s="4" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
@@ -6505,13 +6449,13 @@
     <row r="200" spans="3:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C200" s="1"/>
       <c r="E200" s="1" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="F200" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G200" s="2" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
     </row>
     <row r="201" spans="3:7" x14ac:dyDescent="0.3">
@@ -6563,12 +6507,12 @@
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:C200">
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="notEqual">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="notEqual">
       <formula>F4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F4:G200">
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="notEqual">
+    <cfRule type="cellIs" dxfId="2" priority="5" operator="notEqual">
       <formula>B4</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>